<commit_message>
Add specific cost R$/kWh metrics to FPT pipeline
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,47 +459,67 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Diesel_Custo_R_kWh</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>E94H6_Custo_R_kWh</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Economia_vs_Diesel_R_kWh</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
       </c>
     </row>
@@ -533,31 +553,43 @@
         <v>138.8806565064478</v>
       </c>
       <c r="I2" t="n">
+        <v>1.367320490870933</v>
+      </c>
+      <c r="J2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>100.54</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>40.794</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
+        <v>1.053242035652716</v>
+      </c>
+      <c r="Q2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>-23.75255350293668</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-0.3140784552182163</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-22.97036117831891</v>
       </c>
     </row>
     <row r="3">
@@ -590,31 +622,43 @@
         <v>152.3268464243845</v>
       </c>
       <c r="I3" t="n">
+        <v>1.349845689446515</v>
+      </c>
+      <c r="J3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>43.955</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
+        <v>1.032110516818226</v>
+      </c>
+      <c r="Q3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>-25.09641461978385</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-0.3177351726282893</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-23.53862927536348</v>
       </c>
     </row>
     <row r="4">
@@ -647,31 +691,43 @@
         <v>167.2227432590856</v>
       </c>
       <c r="I4" t="n">
+        <v>1.320738085230403</v>
+      </c>
+      <c r="J4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>47.414</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
+        <v>1.005068185535696</v>
+      </c>
+      <c r="Q4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>-26.39928644672269</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-0.3156698996947078</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-23.90102195316334</v>
       </c>
     </row>
     <row r="5">
@@ -704,31 +760,43 @@
         <v>183.9988276670574</v>
       </c>
       <c r="I5" t="n">
+        <v>1.295256498794189</v>
+      </c>
+      <c r="J5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>135.548</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>51.639</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
+        <v>0.9889070718310762</v>
+      </c>
+      <c r="Q5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>-27.14933161687878</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-0.3063494269631128</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-23.65164175962884</v>
       </c>
     </row>
     <row r="6">
@@ -761,31 +829,43 @@
         <v>208.409613130129</v>
       </c>
       <c r="I6" t="n">
+        <v>1.314863921205991</v>
+      </c>
+      <c r="J6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>58.213</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
+        <v>0.9835344245186554</v>
+      </c>
+      <c r="Q6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>-27.49415690300805</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-0.3313294966873358</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-25.19876706202729</v>
       </c>
     </row>
     <row r="7">
@@ -818,31 +898,43 @@
         <v>219.7983587338804</v>
       </c>
       <c r="I7" t="n">
+        <v>1.30800901886618</v>
+      </c>
+      <c r="J7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>62.66</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
+        <v>0.9820229499329094</v>
+      </c>
+      <c r="Q7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>-25.99914824709473</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-0.3259860689332705</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-24.92231049108856</v>
       </c>
     </row>
     <row r="8">
@@ -875,31 +967,43 @@
         <v>233.694021101993</v>
       </c>
       <c r="I8" t="n">
+        <v>1.306559021984483</v>
+      </c>
+      <c r="J8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>65.848</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
+        <v>0.9810557005390576</v>
+      </c>
+      <c r="Q8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>-26.85818039909983</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-0.3255033214454254</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-24.91302084088255</v>
       </c>
     </row>
     <row r="9">
@@ -932,31 +1036,43 @@
         <v>249.3812426729191</v>
       </c>
       <c r="I9" t="n">
+        <v>1.316127269014794</v>
+      </c>
+      <c r="J9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
+        <v>0.9823210501073268</v>
+      </c>
+      <c r="Q9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>-30.32976437212198</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-0.3338062189074674</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-25.36276139596612</v>
       </c>
     </row>
     <row r="10">
@@ -989,31 +1105,43 @@
         <v>264.7012895662368</v>
       </c>
       <c r="I10" t="n">
+        <v>1.326501688644143</v>
+      </c>
+      <c r="J10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>180.749</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>68.246</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
+        <v>0.9801037970410462</v>
+      </c>
+      <c r="Q10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>-33.07445479329911</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-0.3463978916030965</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-26.11364120894262</v>
       </c>
     </row>
     <row r="11">
@@ -1046,31 +1174,43 @@
         <v>277.2232121922626</v>
       </c>
       <c r="I11" t="n">
+        <v>1.346265262913802</v>
+      </c>
+      <c r="J11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>67.595</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
+        <v>0.9736602111191957</v>
+      </c>
+      <c r="Q11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>-36.70698936277493</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-0.372605051794606</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-27.67694168890273</v>
       </c>
     </row>
     <row r="12">
@@ -1103,31 +1243,43 @@
         <v>256.0347010550997</v>
       </c>
       <c r="I12" t="n">
+        <v>1.342323063096884</v>
+      </c>
+      <c r="J12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>67.64</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
+        <v>0.9955147227280963</v>
+      </c>
+      <c r="Q12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>-31.42346434456669</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-0.3468083403687878</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-25.83642864398556</v>
       </c>
     </row>
     <row r="13">
@@ -1160,31 +1312,43 @@
         <v>246.9882766705745</v>
       </c>
       <c r="I13" t="n">
+        <v>1.371245975843687</v>
+      </c>
+      <c r="J13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>68.863</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
+        <v>1.013090153081947</v>
+      </c>
+      <c r="Q13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>-27.62636731462547</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-0.3581558227617399</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-26.11900629581628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FPT air flow comparison metrics
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,60 +464,80 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Diesel_Air_kg_h</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Diesel_Air_kg_h_kW</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>E94H6_Air_kg_h</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>E94H6_Air_kg_h_kW</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -556,39 +576,51 @@
         <v>1.367320490870933</v>
       </c>
       <c r="J2" t="n">
+        <v>414.5096</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4.080967673971216</v>
+      </c>
+      <c r="L2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>100.54</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>40.794</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
+        <v>343.2376</v>
+      </c>
+      <c r="T2" t="n">
+        <v>3.413940720111398</v>
+      </c>
+      <c r="U2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="R2" t="n">
+      <c r="V2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="S2" t="n">
+      <c r="W2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="T2" t="n">
+      <c r="X2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="U2" t="n">
+      <c r="Y2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -625,39 +657,51 @@
         <v>1.349845689446515</v>
       </c>
       <c r="J3" t="n">
+        <v>472.7576</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4.189345630744473</v>
+      </c>
+      <c r="L3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
         <v>43.955</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
+        <v>368.078</v>
+      </c>
+      <c r="T3" t="n">
+        <v>3.329561233304839</v>
+      </c>
+      <c r="U3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="R3" t="n">
+      <c r="V3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="S3" t="n">
+      <c r="W3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="T3" t="n">
+      <c r="X3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="U3" t="n">
+      <c r="Y3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -694,39 +738,51 @@
         <v>1.320738085230403</v>
       </c>
       <c r="J4" t="n">
+        <v>538.8533</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4.255904799740311</v>
+      </c>
+      <c r="L4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="M4" t="n">
+      <c r="O4" t="n">
         <v>47.414</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
+        <v>404.4934</v>
+      </c>
+      <c r="T4" t="n">
+        <v>3.303159897596289</v>
+      </c>
+      <c r="U4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="R4" t="n">
+      <c r="V4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="S4" t="n">
+      <c r="W4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="T4" t="n">
+      <c r="X4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="U4" t="n">
+      <c r="Y4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -763,39 +819,51 @@
         <v>1.295256498794189</v>
       </c>
       <c r="J5" t="n">
+        <v>611.21</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4.302602003859044</v>
+      </c>
+      <c r="L5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>135.548</v>
       </c>
-      <c r="M5" t="n">
+      <c r="O5" t="n">
         <v>51.639</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
+        <v>439.0808</v>
+      </c>
+      <c r="T5" t="n">
+        <v>3.239301206952519</v>
+      </c>
+      <c r="U5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="R5" t="n">
+      <c r="V5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="S5" t="n">
+      <c r="W5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="T5" t="n">
+      <c r="X5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="U5" t="n">
+      <c r="Y5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -832,39 +900,51 @@
         <v>1.314863921205991</v>
       </c>
       <c r="J6" t="n">
+        <v>717.2952</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4.525441821847942</v>
+      </c>
+      <c r="L6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
         <v>58.213</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
+        <v>493.4668</v>
+      </c>
+      <c r="T6" t="n">
+        <v>3.211861058625126</v>
+      </c>
+      <c r="U6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="R6" t="n">
+      <c r="V6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="S6" t="n">
+      <c r="W6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="T6" t="n">
+      <c r="X6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="U6" t="n">
+      <c r="Y6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -901,39 +981,51 @@
         <v>1.30800901886618</v>
       </c>
       <c r="J7" t="n">
+        <v>759.0008</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4.516775727741662</v>
+      </c>
+      <c r="L7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="M7" t="n">
+      <c r="O7" t="n">
         <v>62.66</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
+        <v>522.3481</v>
+      </c>
+      <c r="T7" t="n">
+        <v>3.153700834751151</v>
+      </c>
+      <c r="U7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="R7" t="n">
+      <c r="V7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="S7" t="n">
+      <c r="W7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="T7" t="n">
+      <c r="X7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="U7" t="n">
+      <c r="Y7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -970,39 +1062,51 @@
         <v>1.306559021984483</v>
       </c>
       <c r="J8" t="n">
+        <v>802.591</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.487202997614924</v>
+      </c>
+      <c r="L8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="L8" t="n">
+      <c r="N8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="M8" t="n">
+      <c r="O8" t="n">
         <v>65.848</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
+        <v>548.4717000000001</v>
+      </c>
+      <c r="T8" t="n">
+        <v>3.14799857887937</v>
+      </c>
+      <c r="U8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="R8" t="n">
+      <c r="V8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="S8" t="n">
+      <c r="W8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="T8" t="n">
+      <c r="X8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="U8" t="n">
+      <c r="Y8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1039,39 +1143,51 @@
         <v>1.316127269014794</v>
       </c>
       <c r="J9" t="n">
+        <v>861.736</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4.547873112410683</v>
+      </c>
+      <c r="L9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="L9" t="n">
+      <c r="N9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="M9" t="n">
+      <c r="O9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
+        <v>558.4708000000001</v>
+      </c>
+      <c r="T9" t="n">
+        <v>3.157496350455755</v>
+      </c>
+      <c r="U9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="R9" t="n">
+      <c r="V9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="S9" t="n">
+      <c r="W9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="T9" t="n">
+      <c r="X9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="U9" t="n">
+      <c r="Y9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1108,39 +1224,51 @@
         <v>1.326501688644143</v>
       </c>
       <c r="J10" t="n">
+        <v>906.6950000000001</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4.543734753072438</v>
+      </c>
+      <c r="L10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="L10" t="n">
+      <c r="N10" t="n">
         <v>180.749</v>
       </c>
-      <c r="M10" t="n">
+      <c r="O10" t="n">
         <v>68.246</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
+        <v>571.497</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3.161826621447422</v>
+      </c>
+      <c r="U10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="R10" t="n">
+      <c r="V10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="S10" t="n">
+      <c r="W10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="T10" t="n">
+      <c r="X10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="U10" t="n">
+      <c r="Y10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1177,39 +1305,51 @@
         <v>1.346265262913802</v>
       </c>
       <c r="J11" t="n">
+        <v>931.8920000000001</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4.525500655108144</v>
+      </c>
+      <c r="L11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="L11" t="n">
+      <c r="N11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>67.595</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
+        <v>572.1528</v>
+      </c>
+      <c r="T11" t="n">
+        <v>3.174929637488791</v>
+      </c>
+      <c r="U11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="R11" t="n">
+      <c r="V11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="S11" t="n">
+      <c r="W11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="T11" t="n">
+      <c r="X11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="U11" t="n">
+      <c r="Y11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1246,39 +1386,51 @@
         <v>1.342323063096884</v>
       </c>
       <c r="J12" t="n">
+        <v>920.961</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.828357974205725</v>
+      </c>
+      <c r="L12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="K12" t="n">
+      <c r="M12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="L12" t="n">
+      <c r="N12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="M12" t="n">
+      <c r="O12" t="n">
         <v>67.64</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
+        <v>566.0339</v>
+      </c>
+      <c r="T12" t="n">
+        <v>3.209340208243088</v>
+      </c>
+      <c r="U12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="R12" t="n">
+      <c r="V12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="S12" t="n">
+      <c r="W12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="T12" t="n">
+      <c r="X12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="U12" t="n">
+      <c r="Y12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -1315,39 +1467,51 @@
         <v>1.371245975843687</v>
       </c>
       <c r="J13" t="n">
+        <v>930.189</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5.164285285998859</v>
+      </c>
+      <c r="L13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="K13" t="n">
+      <c r="M13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="L13" t="n">
+      <c r="N13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="M13" t="n">
+      <c r="O13" t="n">
         <v>68.863</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
+        <v>570.3287</v>
+      </c>
+      <c r="T13" t="n">
+        <v>3.232336817144408</v>
+      </c>
+      <c r="U13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="R13" t="n">
+      <c r="V13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="S13" t="n">
+      <c r="W13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="T13" t="n">
+      <c r="X13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="U13" t="n">
+      <c r="Y13" t="n">
         <v>-26.11900629581628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FPT intake manifold pressure plots
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y13"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,70 +474,80 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Diesel_P_i_MF_mbar</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>E94H6_P_i_MF_mbar</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -582,45 +592,51 @@
         <v>4.080967673971216</v>
       </c>
       <c r="L2" t="n">
+        <v>855.284</v>
+      </c>
+      <c r="M2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>100.54</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>40.794</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>343.2376</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>3.413940720111398</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
+        <v>614.033</v>
+      </c>
+      <c r="W2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AA2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -663,45 +679,51 @@
         <v>4.189345630744473</v>
       </c>
       <c r="L3" t="n">
+        <v>1001.307</v>
+      </c>
+      <c r="M3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>43.955</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>368.078</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>3.329561233304839</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
+        <v>598.8225</v>
+      </c>
+      <c r="W3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Z3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AA3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -744,45 +766,51 @@
         <v>4.255904799740311</v>
       </c>
       <c r="L4" t="n">
+        <v>1151.256</v>
+      </c>
+      <c r="M4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>47.414</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>404.4934</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>3.303159897596289</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
+        <v>618.6754</v>
+      </c>
+      <c r="W4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Y4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Z4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AA4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -825,45 +853,51 @@
         <v>4.302602003859044</v>
       </c>
       <c r="L5" t="n">
+        <v>1333.037</v>
+      </c>
+      <c r="M5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>135.548</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>51.639</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>439.0808</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>3.239301206952519</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
+        <v>645.2624999999999</v>
+      </c>
+      <c r="W5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Z5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AA5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -906,45 +940,51 @@
         <v>4.525441821847942</v>
       </c>
       <c r="L6" t="n">
+        <v>1638.823</v>
+      </c>
+      <c r="M6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>58.213</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>493.4668</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>3.211861058625126</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
+        <v>706.9007</v>
+      </c>
+      <c r="W6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="W6" t="n">
+      <c r="Y6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Z6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AA6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -987,45 +1027,51 @@
         <v>4.516775727741662</v>
       </c>
       <c r="L7" t="n">
+        <v>1713.213</v>
+      </c>
+      <c r="M7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>62.66</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>522.3481</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>3.153700834751151</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
+        <v>720.8134</v>
+      </c>
+      <c r="W7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="W7" t="n">
+      <c r="Y7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Z7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AA7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -1068,45 +1114,51 @@
         <v>4.487202997614924</v>
       </c>
       <c r="L8" t="n">
+        <v>1772.888</v>
+      </c>
+      <c r="M8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>65.848</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>548.4717000000001</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>3.14799857887937</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
+        <v>714.4274</v>
+      </c>
+      <c r="W8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="W8" t="n">
+      <c r="Y8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Z8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AA8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1149,45 +1201,51 @@
         <v>4.547873112410683</v>
       </c>
       <c r="L9" t="n">
+        <v>1888.707</v>
+      </c>
+      <c r="M9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>558.4708000000001</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>3.157496350455755</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
+        <v>665.6324</v>
+      </c>
+      <c r="W9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="W9" t="n">
+      <c r="Y9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Z9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AA9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1230,45 +1288,51 @@
         <v>4.543734753072438</v>
       </c>
       <c r="L10" t="n">
+        <v>1963.644</v>
+      </c>
+      <c r="M10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>180.749</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>68.246</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>571.497</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>3.161826621447422</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
+        <v>635.0775</v>
+      </c>
+      <c r="W10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="W10" t="n">
+      <c r="Y10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Z10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AA10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1311,45 +1375,51 @@
         <v>4.525500655108144</v>
       </c>
       <c r="L11" t="n">
+        <v>1970.661</v>
+      </c>
+      <c r="M11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>67.595</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>572.1528</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>3.174929637488791</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
+        <v>574.5626999999999</v>
+      </c>
+      <c r="W11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="W11" t="n">
+      <c r="Y11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Z11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AA11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1392,45 +1462,51 @@
         <v>4.828357974205725</v>
       </c>
       <c r="L12" t="n">
+        <v>1838.046</v>
+      </c>
+      <c r="M12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>67.64</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>566.0339</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>3.209340208243088</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
+        <v>543.4535999999999</v>
+      </c>
+      <c r="W12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="W12" t="n">
+      <c r="Y12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Z12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AA12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -1473,45 +1549,51 @@
         <v>5.164285285998859</v>
       </c>
       <c r="L13" t="n">
+        <v>1783.737</v>
+      </c>
+      <c r="M13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>68.863</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>570.3287</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>3.232336817144408</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
+        <v>546.0051999999999</v>
+      </c>
+      <c r="W13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="V13" t="n">
+      <c r="X13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="W13" t="n">
+      <c r="Y13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Z13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AA13" t="n">
         <v>-26.11900629581628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FPT volumetric efficiency and intercooler power
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,75 +479,95 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Diesel_Eta_v_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Diesel_Q_intercooler_kW</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>E94H6_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>E94H6_Eta_v_pct</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>E94H6_Q_intercooler_kW</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -595,48 +615,60 @@
         <v>855.284</v>
       </c>
       <c r="M2" t="n">
+        <v>85.76093459672069</v>
+      </c>
+      <c r="N2" t="n">
+        <v>7.371469710110599</v>
+      </c>
+      <c r="O2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>100.54</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>40.794</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>343.2376</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>3.413940720111398</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>614.033</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
+        <v>71.93240293527499</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>5.123065851202532</v>
+      </c>
+      <c r="AA2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AC2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AD2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AE2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -682,48 +714,60 @@
         <v>1001.307</v>
       </c>
       <c r="M3" t="n">
+        <v>90.16074520659268</v>
+      </c>
+      <c r="N3" t="n">
+        <v>9.478317989122266</v>
+      </c>
+      <c r="O3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>43.955</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>368.078</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>3.329561233304839</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>598.8225</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
+        <v>70.63183398702874</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>5.277530107879249</v>
+      </c>
+      <c r="AA3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AB3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AC3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -769,48 +813,60 @@
         <v>1151.256</v>
       </c>
       <c r="M4" t="n">
+        <v>94.87618551787044</v>
+      </c>
+      <c r="N4" t="n">
+        <v>12.20416552876442</v>
+      </c>
+      <c r="O4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>47.414</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>404.4934</v>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>3.303159897596289</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>618.6754</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Y4" t="n">
+        <v>71.49738164776328</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>5.953061266356182</v>
+      </c>
+      <c r="AA4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AC4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AD4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AE4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -856,48 +912,60 @@
         <v>1333.037</v>
       </c>
       <c r="M5" t="n">
+        <v>100.0868527420609</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15.7296847843975</v>
+      </c>
+      <c r="O5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>135.548</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>51.639</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="T5" t="n">
+      <c r="V5" t="n">
         <v>439.0808</v>
       </c>
-      <c r="U5" t="n">
+      <c r="W5" t="n">
         <v>3.239301206952519</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>645.2624999999999</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="n">
+        <v>72.01830624666327</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>6.691189980673633</v>
+      </c>
+      <c r="AA5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AC5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AD5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AE5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -943,48 +1011,60 @@
         <v>1638.823</v>
       </c>
       <c r="M6" t="n">
+        <v>109.7015870271678</v>
+      </c>
+      <c r="N6" t="n">
+        <v>22.0044045378286</v>
+      </c>
+      <c r="O6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>58.213</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>493.4668</v>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>3.211861058625126</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>706.9007</v>
       </c>
-      <c r="W6" t="n">
+      <c r="Y6" t="n">
+        <v>75.58050048948876</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>8.086896229873149</v>
+      </c>
+      <c r="AA6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AC6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AD6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AE6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -1030,48 +1110,60 @@
         <v>1713.213</v>
       </c>
       <c r="M7" t="n">
+        <v>108.7813121895017</v>
+      </c>
+      <c r="N7" t="n">
+        <v>24.09184179296887</v>
+      </c>
+      <c r="O7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>62.66</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>522.3481</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>3.153700834751151</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>720.8134</v>
       </c>
-      <c r="W7" t="n">
+      <c r="Y7" t="n">
+        <v>74.81759260933984</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>8.844545266070686</v>
+      </c>
+      <c r="AA7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AC7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AD7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AE7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -1117,48 +1209,60 @@
         <v>1772.888</v>
       </c>
       <c r="M8" t="n">
+        <v>108.2178545232641</v>
+      </c>
+      <c r="N8" t="n">
+        <v>26.15586071767862</v>
+      </c>
+      <c r="O8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>65.848</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="T8" t="n">
+      <c r="V8" t="n">
         <v>548.4717000000001</v>
       </c>
-      <c r="U8" t="n">
+      <c r="W8" t="n">
         <v>3.14799857887937</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>714.4274</v>
       </c>
-      <c r="W8" t="n">
+      <c r="Y8" t="n">
+        <v>73.92228427959083</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>9.2689338761061</v>
+      </c>
+      <c r="AA8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AB8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AC8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AD8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AE8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1204,48 +1308,60 @@
         <v>1888.707</v>
       </c>
       <c r="M9" t="n">
+        <v>109.7248753354082</v>
+      </c>
+      <c r="N9" t="n">
+        <v>29.65123841101533</v>
+      </c>
+      <c r="O9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="S9" t="n">
+      <c r="U9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="T9" t="n">
+      <c r="V9" t="n">
         <v>558.4708000000001</v>
       </c>
-      <c r="U9" t="n">
+      <c r="W9" t="n">
         <v>3.157496350455755</v>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
         <v>665.6324</v>
       </c>
-      <c r="W9" t="n">
+      <c r="Y9" t="n">
+        <v>70.97223581427968</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>9.008301684857699</v>
+      </c>
+      <c r="AA9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AB9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AC9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AD9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AE9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1291,48 +1407,60 @@
         <v>1963.644</v>
       </c>
       <c r="M10" t="n">
+        <v>109.4746178509552</v>
+      </c>
+      <c r="N10" t="n">
+        <v>32.24423217187896</v>
+      </c>
+      <c r="O10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>180.749</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>68.246</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="T10" t="n">
+      <c r="V10" t="n">
         <v>571.497</v>
       </c>
-      <c r="U10" t="n">
+      <c r="W10" t="n">
         <v>3.161826621447422</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>635.0775</v>
       </c>
-      <c r="W10" t="n">
+      <c r="Y10" t="n">
+        <v>69.18864744169888</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>8.637737840493624</v>
+      </c>
+      <c r="AA10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AB10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AC10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AD10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AE10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1378,48 +1506,60 @@
         <v>1970.661</v>
       </c>
       <c r="M11" t="n">
+        <v>106.7553373802408</v>
+      </c>
+      <c r="N11" t="n">
+        <v>33.38365515560616</v>
+      </c>
+      <c r="O11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>67.595</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="S11" t="n">
+      <c r="U11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="T11" t="n">
+      <c r="V11" t="n">
         <v>572.1528</v>
       </c>
-      <c r="U11" t="n">
+      <c r="W11" t="n">
         <v>3.174929637488791</v>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
         <v>574.5626999999999</v>
       </c>
-      <c r="W11" t="n">
+      <c r="Y11" t="n">
+        <v>65.32181088310659</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>8.353255586685897</v>
+      </c>
+      <c r="AA11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AB11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AC11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AD11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AE11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1465,48 +1605,60 @@
         <v>1838.046</v>
       </c>
       <c r="M12" t="n">
+        <v>100.6382935248363</v>
+      </c>
+      <c r="N12" t="n">
+        <v>31.04210160607312</v>
+      </c>
+      <c r="O12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>67.64</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="R12" t="n">
+      <c r="T12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="T12" t="n">
+      <c r="V12" t="n">
         <v>566.0339</v>
       </c>
-      <c r="U12" t="n">
+      <c r="W12" t="n">
         <v>3.209340208243088</v>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
         <v>543.4535999999999</v>
       </c>
-      <c r="W12" t="n">
+      <c r="Y12" t="n">
+        <v>61.61609472600434</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>7.81562819139441</v>
+      </c>
+      <c r="AA12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="X12" t="n">
+      <c r="AB12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AC12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AD12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AE12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -1552,48 +1704,60 @@
         <v>1783.737</v>
       </c>
       <c r="M13" t="n">
+        <v>96.93582851694275</v>
+      </c>
+      <c r="N13" t="n">
+        <v>30.86135953909287</v>
+      </c>
+      <c r="O13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>68.863</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="R13" t="n">
+      <c r="T13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="S13" t="n">
+      <c r="U13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="T13" t="n">
+      <c r="V13" t="n">
         <v>570.3287</v>
       </c>
-      <c r="U13" t="n">
+      <c r="W13" t="n">
         <v>3.232336817144408</v>
       </c>
-      <c r="V13" t="n">
+      <c r="X13" t="n">
         <v>546.0051999999999</v>
       </c>
-      <c r="W13" t="n">
+      <c r="Y13" t="n">
+        <v>59.72376574394802</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>7.498332516326033</v>
+      </c>
+      <c r="AA13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="X13" t="n">
+      <c r="AB13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AC13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AD13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AE13" t="n">
         <v>-26.11900629581628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FPT compressor pressure ratio curves
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI13"/>
+  <dimension ref="A1:AM13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,110 +484,130 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Diesel_Compressor_PRatio_abs</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Diesel_Compressor_VolFlow_m3_s</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>Diesel_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Diesel_Eta_v_pct</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Diesel_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>E94H6_Torque_Nm</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>E94H6_BMEP_bar</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>E94H6_Compressor_PRatio_abs</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>E94H6_Compressor_VolFlow_m3_s</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
         <is>
           <t>E94H6_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>E94H6_Eta_v_pct</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>E94H6_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -638,69 +658,81 @@
         <v>4.080967673971216</v>
       </c>
       <c r="N2" t="n">
+        <v>1.830054878769283</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.09816014520570203</v>
+      </c>
+      <c r="P2" t="n">
         <v>855.284</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>165.1217994474175</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>7.371469710110599</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>100.54</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>40.794</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
         <v>872.4690000000001</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AA2" t="n">
         <v>16.36383403513333</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AB2" t="n">
         <v>343.2376</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AC2" t="n">
         <v>3.413940720111398</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AD2" t="n">
+        <v>1.639548038862097</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0.08409867297052714</v>
+      </c>
+      <c r="AF2" t="n">
         <v>614.033</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AG2" t="n">
         <v>138.4967160992609</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AH2" t="n">
         <v>5.123065851202532</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AI2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AJ2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AK2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AL2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AM2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -749,69 +781,81 @@
         <v>4.189345630744473</v>
       </c>
       <c r="N3" t="n">
+        <v>1.978027048534528</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.1121661376558138</v>
+      </c>
+      <c r="P3" t="n">
         <v>1001.307</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>173.5930765917979</v>
       </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
         <v>9.478317989122266</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>43.955</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Z3" t="n">
         <v>880.187</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AA3" t="n">
         <v>16.50859112229994</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AB3" t="n">
         <v>368.078</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AC3" t="n">
         <v>3.329561233304839</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AD3" t="n">
+        <v>1.630077448476151</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.09032687829722572</v>
+      </c>
+      <c r="AF3" t="n">
         <v>598.8225</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AG3" t="n">
         <v>135.9926355869658</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AH3" t="n">
         <v>5.277530107879249</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AI3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AJ3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AK3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AL3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AM3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -860,69 +904,81 @@
         <v>4.255904799740311</v>
       </c>
       <c r="N4" t="n">
+        <v>2.131624829845151</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.1282266582516197</v>
+      </c>
+      <c r="P4" t="n">
         <v>1151.256</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>182.672058683661</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>12.20416552876442</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>47.414</v>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Y4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Z4" t="n">
         <v>898.739</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AA4" t="n">
         <v>16.85654829787843</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AB4" t="n">
         <v>404.4934</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AC4" t="n">
         <v>3.303159897596289</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AD4" t="n">
+        <v>1.659473125376284</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.09950172123356095</v>
+      </c>
+      <c r="AF4" t="n">
         <v>618.6754</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AG4" t="n">
         <v>137.6591377994248</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AH4" t="n">
         <v>5.953061266356182</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AI4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AJ4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AK4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="AL4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="AM4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -971,69 +1027,81 @@
         <v>4.302602003859044</v>
       </c>
       <c r="N5" t="n">
+        <v>2.316668221592714</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.1457178337499356</v>
+      </c>
+      <c r="P5" t="n">
         <v>1333.037</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>192.7045373690426</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>15.7296847843975</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>135.548</v>
       </c>
-      <c r="T5" t="n">
+      <c r="V5" t="n">
         <v>51.639</v>
       </c>
-      <c r="U5" t="n">
+      <c r="W5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Z5" t="n">
         <v>924.303</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AA5" t="n">
         <v>17.33602098203586</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AB5" t="n">
         <v>439.0808</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AC5" t="n">
         <v>3.239301206952519</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AD5" t="n">
+        <v>1.695440603825862</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.1083561955826871</v>
+      </c>
+      <c r="AF5" t="n">
         <v>645.2624999999999</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AG5" t="n">
         <v>138.6621120271576</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AH5" t="n">
         <v>6.691189980673633</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AI5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AJ5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AK5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="AL5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AM5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -1082,69 +1150,81 @@
         <v>4.525441821847942</v>
       </c>
       <c r="N6" t="n">
+        <v>2.626861387706466</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.1715072063519566</v>
+      </c>
+      <c r="P6" t="n">
         <v>1638.823</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>211.2164884552933</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>22.0044045378286</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="S6" t="n">
+      <c r="U6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>58.213</v>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="W6" t="n">
+      <c r="Y6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Z6" t="n">
         <v>977.721</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AA6" t="n">
         <v>18.33791707976398</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AB6" t="n">
         <v>493.4668</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AC6" t="n">
         <v>3.211861058625126</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AD6" t="n">
+        <v>1.770896081789997</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.1222650200064994</v>
+      </c>
+      <c r="AF6" t="n">
         <v>706.9007</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AG6" t="n">
         <v>145.520665121553</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AH6" t="n">
         <v>8.086896229873149</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AI6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AJ6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AK6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AL6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AM6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -1193,69 +1273,81 @@
         <v>4.516775727741662</v>
       </c>
       <c r="N7" t="n">
+        <v>2.708530721619916</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.1820273138810209</v>
+      </c>
+      <c r="P7" t="n">
         <v>1713.213</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>209.4446160066526</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>24.09184179296887</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="S7" t="n">
+      <c r="U7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>62.66</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="W7" t="n">
+      <c r="Y7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Z7" t="n">
         <v>988.704</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="AA7" t="n">
         <v>18.54391177895428</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AB7" t="n">
         <v>522.3481</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AC7" t="n">
         <v>3.153700834751151</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AD7" t="n">
+        <v>1.796419241697494</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.1299030882458023</v>
+      </c>
+      <c r="AF7" t="n">
         <v>720.8134</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AG7" t="n">
         <v>144.0517827851469</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AH7" t="n">
         <v>8.844545266070686</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AI7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AJ7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AK7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AL7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AM7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -1304,69 +1396,81 @@
         <v>4.487202997614924</v>
       </c>
       <c r="N8" t="n">
+        <v>2.774061961611681</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.1928176157700011</v>
+      </c>
+      <c r="P8" t="n">
         <v>1772.888</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>208.3597497537472</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>26.15586071767862</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="S8" t="n">
+      <c r="U8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="T8" t="n">
+      <c r="V8" t="n">
         <v>65.848</v>
       </c>
-      <c r="U8" t="n">
+      <c r="W8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="W8" t="n">
+      <c r="Y8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Z8" t="n">
         <v>978.561</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AA8" t="n">
         <v>18.35367193247452</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AB8" t="n">
         <v>548.4717000000001</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AC8" t="n">
         <v>3.14799857887937</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AD8" t="n">
+        <v>1.798899826954319</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0.1367244366904898</v>
+      </c>
+      <c r="AF8" t="n">
         <v>714.4274</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AG8" t="n">
         <v>142.3279801801077</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AH8" t="n">
         <v>9.2689338761061</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AI8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AJ8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AK8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="AL8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="AM8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1415,69 +1519,81 @@
         <v>4.547873112410683</v>
       </c>
       <c r="N9" t="n">
+        <v>2.899580384839584</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.2076704395240223</v>
+      </c>
+      <c r="P9" t="n">
         <v>1888.707</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>211.2613271383233</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>29.65123841101533</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="S9" t="n">
+      <c r="U9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="T9" t="n">
+      <c r="V9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="U9" t="n">
+      <c r="W9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="W9" t="n">
+      <c r="Y9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Z9" t="n">
         <v>938.7430000000001</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AA9" t="n">
         <v>17.60685440244086</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AB9" t="n">
         <v>558.4708000000001</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AC9" t="n">
         <v>3.157496350455755</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AD9" t="n">
+        <v>1.753481773347166</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.1393656804799396</v>
+      </c>
+      <c r="AF9" t="n">
         <v>665.6324</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AG9" t="n">
         <v>136.6480361200311</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AH9" t="n">
         <v>9.008301684857699</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AI9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AJ9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AK9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="AL9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AM9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1526,69 +1642,81 @@
         <v>4.543734753072438</v>
       </c>
       <c r="N10" t="n">
+        <v>2.983147722347778</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.2191140155571194</v>
+      </c>
+      <c r="P10" t="n">
         <v>1963.644</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>210.7794881010929</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>32.24423217187896</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="S10" t="n">
+      <c r="U10" t="n">
         <v>180.749</v>
       </c>
-      <c r="T10" t="n">
+      <c r="V10" t="n">
         <v>68.246</v>
       </c>
-      <c r="U10" t="n">
+      <c r="W10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="W10" t="n">
+      <c r="Y10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Z10" t="n">
         <v>907.992</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AA10" t="n">
         <v>17.03009550279584</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AB10" t="n">
         <v>571.497</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AC10" t="n">
         <v>3.161826621447422</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AD10" t="n">
+        <v>1.727460748434112</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.1427916285441307</v>
+      </c>
+      <c r="AF10" t="n">
         <v>635.0775</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AG10" t="n">
         <v>133.2139629847635</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AH10" t="n">
         <v>8.637737840493624</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AI10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AJ10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AK10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="AL10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AM10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1637,69 +1765,81 @@
         <v>4.525500655108144</v>
       </c>
       <c r="N11" t="n">
+        <v>2.994461657843572</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.2254507137664753</v>
+      </c>
+      <c r="P11" t="n">
         <v>1970.661</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>205.5438585380755</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>33.38365515560616</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="S11" t="n">
+      <c r="U11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="T11" t="n">
+      <c r="V11" t="n">
         <v>67.595</v>
       </c>
-      <c r="U11" t="n">
+      <c r="W11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="W11" t="n">
+      <c r="Y11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Z11" t="n">
         <v>860.047</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AA11" t="n">
         <v>16.13084977278771</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AB11" t="n">
         <v>572.1528</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AC11" t="n">
         <v>3.174929637488791</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AD11" t="n">
+        <v>1.66796685740581</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.1429858246464122</v>
+      </c>
+      <c r="AF11" t="n">
         <v>574.5626999999999</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AG11" t="n">
         <v>125.7688597600112</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AH11" t="n">
         <v>8.353255586685897</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AI11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AJ11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AK11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="AL11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="AM11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1748,69 +1888,81 @@
         <v>4.828357974205725</v>
       </c>
       <c r="N12" t="n">
+        <v>2.860976546474551</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.2227259593366687</v>
+      </c>
+      <c r="P12" t="n">
         <v>1838.046</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>193.7662666373713</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>31.04210160607312</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="S12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="R12" t="n">
+      <c r="T12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="S12" t="n">
+      <c r="U12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="T12" t="n">
+      <c r="V12" t="n">
         <v>67.64</v>
       </c>
-      <c r="U12" t="n">
+      <c r="W12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="W12" t="n">
+      <c r="Y12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Z12" t="n">
         <v>801.8111</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AA12" t="n">
         <v>15.03859021687613</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AB12" t="n">
         <v>566.0339</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AC12" t="n">
         <v>3.209340208243088</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AD12" t="n">
+        <v>1.634463357608077</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.141379834838291</v>
+      </c>
+      <c r="AF12" t="n">
         <v>543.4535999999999</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AG12" t="n">
         <v>118.63397342768</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AH12" t="n">
         <v>7.81562819139441</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AI12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AJ12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AK12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="AH12" t="n">
+      <c r="AL12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="AM12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -1859,69 +2011,81 @@
         <v>5.164285285998859</v>
       </c>
       <c r="N13" t="n">
+        <v>2.809971531120575</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.2252061520225796</v>
+      </c>
+      <c r="P13" t="n">
         <v>1783.737</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>186.6376399803823</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>30.86135953909287</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="S13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="R13" t="n">
+      <c r="T13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="S13" t="n">
+      <c r="U13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="T13" t="n">
+      <c r="V13" t="n">
         <v>68.863</v>
       </c>
-      <c r="U13" t="n">
+      <c r="W13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="V13" t="n">
+      <c r="X13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="W13" t="n">
+      <c r="Y13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Z13" t="n">
         <v>765.7402</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AA13" t="n">
         <v>14.36205245897539</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AB13" t="n">
         <v>570.3287</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AC13" t="n">
         <v>3.232336817144408</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AD13" t="n">
+        <v>1.638711519816756</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.14247457554881</v>
+      </c>
+      <c r="AF13" t="n">
         <v>546.0051999999999</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AG13" t="n">
         <v>114.9905340443179</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AH13" t="n">
         <v>7.498332516326033</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AI13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AJ13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AK13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="AL13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AM13" t="n">
         <v>-26.11900629581628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add corrected volumetric efficiency to FPT outputs
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM13"/>
+  <dimension ref="A1:AO13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,110 +504,120 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
+          <t>Diesel_Eta_v_corr_press_pct</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>Diesel_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Diesel_n_th_pct</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>E94H6_Speed_RPM</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>E94H6_Power_kW</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_kg_h</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>E94H6_Consumo_L_h</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_h</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>E94H6_Custo_R_kWh</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>E94H6_Torque_Nm</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>E94H6_BMEP_bar</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>E94H6_Air_kg_h_kW</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>E94H6_Compressor_PRatio_abs</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>E94H6_Compressor_VolFlow_m3_s</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>E94H6_P_i_MF_mbar</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>E94H6_Eta_v_pct</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>E94H6_Eta_v_corr_press_pct</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>E94H6_Q_intercooler_kW</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>E94H6_n_th_pct</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_h</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_pct</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
@@ -670,69 +680,75 @@
         <v>165.1217994474175</v>
       </c>
       <c r="R2" t="n">
+        <v>89.53049046089023</v>
+      </c>
+      <c r="S2" t="n">
         <v>7.371469710110599</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>40.06670021108439</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>1099.978</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>100.54</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>40.794</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>50.42521631644005</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>105.8929542645241</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>1.053242035652716</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>872.4690000000001</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>16.36383403513333</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>343.2376</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>3.413940720111398</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>1.639548038862097</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>0.08409867297052714</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
         <v>614.033</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AH2" t="n">
         <v>138.4967160992609</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
+        <v>86.22884318176169</v>
+      </c>
+      <c r="AJ2" t="n">
         <v>5.123065851202532</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AK2" t="n">
         <v>36.06699694000912</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AL2" t="n">
         <v>-32.98770224192374</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AM2" t="n">
         <v>-23.75255350293668</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AN2" t="n">
         <v>-0.3140784552182163</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="AO2" t="n">
         <v>-22.97036117831891</v>
       </c>
     </row>
@@ -793,69 +809,75 @@
         <v>173.5930765917979</v>
       </c>
       <c r="R3" t="n">
+        <v>87.30038995420821</v>
+      </c>
+      <c r="S3" t="n">
         <v>9.478317989122266</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>40.58539478143002</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>1199.915</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>110.5485</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>43.955</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>54.33250927070458</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>114.0982694684796</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>1.032110516818226</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>880.187</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>16.50859112229994</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>368.078</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>3.329561233304839</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>1.630077448476151</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>0.09032687829722572</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="n">
         <v>598.8225</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AH3" t="n">
         <v>135.9926355869658</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
+        <v>85.46880307825234</v>
+      </c>
+      <c r="AJ3" t="n">
         <v>5.277530107879249</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AK3" t="n">
         <v>36.80543571446407</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AL3" t="n">
         <v>-38.22857695590493</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AM3" t="n">
         <v>-25.09641461978385</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AN3" t="n">
         <v>-0.3177351726282893</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AO3" t="n">
         <v>-23.53862927536348</v>
       </c>
     </row>
@@ -916,69 +938,75 @@
         <v>182.672058683661</v>
       </c>
       <c r="R4" t="n">
+        <v>85.50134339308684</v>
+      </c>
+      <c r="S4" t="n">
         <v>12.20416552876442</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>41.47985191980082</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>1299.975</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>122.4565</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>47.414</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>58.60815822002472</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>123.0771322620519</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>1.005068185535696</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>898.739</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>16.85654829787843</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>404.4934</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>3.303159897596289</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>1.659473125376284</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AF4" t="n">
         <v>0.09950172123356095</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>618.6754</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AH4" t="n">
         <v>137.6591377994248</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="AI4" t="n">
+        <v>85.46350983217454</v>
+      </c>
+      <c r="AJ4" t="n">
         <v>5.953061266356182</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="AK4" t="n">
         <v>37.79572154771618</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AL4" t="n">
         <v>-44.14561099703366</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="AM4" t="n">
         <v>-26.39928644672269</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AN4" t="n">
         <v>-0.3156698996947078</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="AO4" t="n">
         <v>-23.90102195316334</v>
       </c>
     </row>
@@ -1039,69 +1067,75 @@
         <v>192.7045373690426</v>
       </c>
       <c r="R5" t="n">
+        <v>83.20827691755936</v>
+      </c>
+      <c r="S5" t="n">
         <v>15.7296847843975</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>42.29588521748337</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>1399.957</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>135.548</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>51.639</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>63.83065512978986</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>134.0443757725587</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>0.9889070718310762</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>924.303</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>17.33602098203586</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>439.0808</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>3.239301206952519</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>1.695440603825862</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>0.1083561955826871</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AG5" t="n">
         <v>645.2624999999999</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AH5" t="n">
         <v>138.6621120271576</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="AI5" t="n">
+        <v>84.70596150097511</v>
+      </c>
+      <c r="AJ5" t="n">
         <v>6.691189980673633</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AK5" t="n">
         <v>38.41339430067745</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AL5" t="n">
         <v>-49.95445189449873</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="AM5" t="n">
         <v>-27.14933161687878</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="AN5" t="n">
         <v>-0.3063494269631128</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="AO5" t="n">
         <v>-23.65164175962884</v>
       </c>
     </row>
@@ -1162,69 +1196,75 @@
         <v>211.2164884552933</v>
       </c>
       <c r="R6" t="n">
+        <v>80.68498644336826</v>
+      </c>
+      <c r="S6" t="n">
         <v>22.0044045378286</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>41.6651634565732</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>1499.988</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>153.6389</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>58.213</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>71.95673671199012</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>151.1091470951793</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>0.9835344245186554</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>977.721</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>18.33791707976398</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>493.4668</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>3.211861058625126</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>1.770896081789997</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>0.1222650200064994</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AG6" t="n">
         <v>706.9007</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AH6" t="n">
         <v>145.520665121553</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
+        <v>85.70985160255658</v>
+      </c>
+      <c r="AJ6" t="n">
         <v>8.086896229873149</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AK6" t="n">
         <v>38.62323100237857</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AL6" t="n">
         <v>-57.30046603494972</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AM6" t="n">
         <v>-27.49415690300805</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AN6" t="n">
         <v>-0.3313294966873358</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AO6" t="n">
         <v>-25.19876706202729</v>
       </c>
     </row>
@@ -1285,69 +1325,75 @@
         <v>209.4446160066526</v>
       </c>
       <c r="R7" t="n">
+        <v>77.82495205427415</v>
+      </c>
+      <c r="S7" t="n">
         <v>24.09184179296887</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>41.8835186990429</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>1600.025</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>165.6302</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>62.66</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>77.45364647713227</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>162.6526576019778</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>0.9820229499329094</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>988.704</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>18.54391177895428</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>522.3481</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>3.153700834751151</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>1.796419241697494</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AF7" t="n">
         <v>0.1299030882458023</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AG7" t="n">
         <v>720.8134</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AH7" t="n">
         <v>144.0517827851469</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AI7" t="n">
+        <v>84.16387597497736</v>
+      </c>
+      <c r="AJ7" t="n">
         <v>8.844545266070686</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AK7" t="n">
         <v>38.68267771091372</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AL7" t="n">
         <v>-57.14570113190265</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="AM7" t="n">
         <v>-25.99914824709473</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="AN7" t="n">
         <v>-0.3259860689332705</v>
       </c>
-      <c r="AM7" t="n">
+      <c r="AO7" t="n">
         <v>-24.92231049108856</v>
       </c>
     </row>
@@ -1408,69 +1454,75 @@
         <v>208.3597497537472</v>
       </c>
       <c r="R8" t="n">
+        <v>75.76342857306034</v>
+      </c>
+      <c r="S8" t="n">
         <v>26.15586071767862</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>41.93000031256837</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>1699.985</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>174.2287</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>65.848</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>81.39431396786156</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>170.9280593325093</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>0.9810557005390576</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>978.561</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>18.35367193247452</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>548.4717000000001</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>3.14799857887937</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>1.798899826954319</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AF8" t="n">
         <v>0.1367244366904898</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AG8" t="n">
         <v>714.4274</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AH8" t="n">
         <v>142.3279801801077</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="AI8" t="n">
+        <v>83.46414090829468</v>
+      </c>
+      <c r="AJ8" t="n">
         <v>9.2689338761061</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="AK8" t="n">
         <v>38.72081601085723</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AL8" t="n">
         <v>-62.76596176948371</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AM8" t="n">
         <v>-26.85818039909983</v>
       </c>
-      <c r="AL8" t="n">
+      <c r="AN8" t="n">
         <v>-0.3255033214454254</v>
       </c>
-      <c r="AM8" t="n">
+      <c r="AO8" t="n">
         <v>-24.91302084088255</v>
       </c>
     </row>
@@ -1531,69 +1583,75 @@
         <v>211.2613271383233</v>
       </c>
       <c r="R9" t="n">
+        <v>73.75235486943424</v>
+      </c>
+      <c r="S9" t="n">
         <v>29.65123841101533</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>41.62516915344194</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>1800.025</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>176.8714</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>66.93300000000001</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>82.73547589616811</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>173.744499381953</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>0.9823210501073268</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>938.7430000000001</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>17.60685440244086</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>558.4708000000001</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>3.157496350455755</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>1.753481773347166</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AF9" t="n">
         <v>0.1393656804799396</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AG9" t="n">
         <v>665.6324</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AH9" t="n">
         <v>136.6480361200311</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="AI9" t="n">
+        <v>82.46264077209011</v>
+      </c>
+      <c r="AJ9" t="n">
         <v>9.008301684857699</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AK9" t="n">
         <v>38.67093886751694</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AL9" t="n">
         <v>-75.63674329096608</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AM9" t="n">
         <v>-30.32976437212198</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="AN9" t="n">
         <v>-0.3338062189074674</v>
       </c>
-      <c r="AM9" t="n">
+      <c r="AO9" t="n">
         <v>-25.36276139596612</v>
       </c>
     </row>
@@ -1654,69 +1712,75 @@
         <v>210.7794881010929</v>
       </c>
       <c r="R10" t="n">
+        <v>71.73166204840319</v>
+      </c>
+      <c r="S10" t="n">
         <v>32.24423217187896</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>41.29962341487465</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>1899.959</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>180.749</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>68.246</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>84.3584672435105</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>177.1527812113721</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>0.9801037970410462</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>907.992</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>17.03009550279584</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>571.497</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>3.161826621447422</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>1.727460748434112</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>0.1427916285441307</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AG10" t="n">
         <v>635.0775</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AH10" t="n">
         <v>133.2139629847635</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="AI10" t="n">
+        <v>81.88070312443769</v>
+      </c>
+      <c r="AJ10" t="n">
         <v>8.637737840493624</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AK10" t="n">
         <v>38.75842272181769</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AL10" t="n">
         <v>-87.54850835486477</v>
       </c>
-      <c r="AK10" t="n">
+      <c r="AM10" t="n">
         <v>-33.07445479329911</v>
       </c>
-      <c r="AL10" t="n">
+      <c r="AN10" t="n">
         <v>-0.3463978916030965</v>
       </c>
-      <c r="AM10" t="n">
+      <c r="AO10" t="n">
         <v>-26.11364120894262</v>
       </c>
     </row>
@@ -1777,69 +1841,75 @@
         <v>205.5438585380755</v>
       </c>
       <c r="R11" t="n">
+        <v>69.7853840295766</v>
+      </c>
+      <c r="S11" t="n">
         <v>33.38365515560616</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>40.69333266582701</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>1999.957</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>180.2096</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>67.595</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>83.55377008652657</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>175.4629171817058</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>0.9736602111191957</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>860.047</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>16.13084977278771</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>572.1528</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>3.174929637488791</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>1.66796685740581</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AF11" t="n">
         <v>0.1429858246464122</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AG11" t="n">
         <v>574.5626999999999</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AH11" t="n">
         <v>125.7688597600112</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="AI11" t="n">
+        <v>80.25122720311542</v>
+      </c>
+      <c r="AJ11" t="n">
         <v>8.353255586685897</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="AK11" t="n">
         <v>39.01492208797374</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AL11" t="n">
         <v>-101.7602950105568</v>
       </c>
-      <c r="AK11" t="n">
+      <c r="AM11" t="n">
         <v>-36.70698936277493</v>
       </c>
-      <c r="AL11" t="n">
+      <c r="AN11" t="n">
         <v>-0.372605051794606</v>
       </c>
-      <c r="AM11" t="n">
+      <c r="AO11" t="n">
         <v>-27.67694168890273</v>
       </c>
     </row>
@@ -1900,69 +1970,75 @@
         <v>193.7662666373713</v>
       </c>
       <c r="R12" t="n">
+        <v>68.84674189881788</v>
+      </c>
+      <c r="S12" t="n">
         <v>31.04210160607312</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>40.81284282921114</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>2099.989</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>176.3708</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>67.64</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>83.60939431396787</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>175.5797280593325</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>0.9955147227280963</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AA12" t="n">
         <v>801.8111</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>15.03859021687613</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>566.0339</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>3.209340208243088</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>1.634463357608077</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>0.141379834838291</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AG12" t="n">
         <v>543.4535999999999</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AH12" t="n">
         <v>118.63397342768</v>
       </c>
-      <c r="AH12" t="n">
+      <c r="AI12" t="n">
+        <v>77.21156292885306</v>
+      </c>
+      <c r="AJ12" t="n">
         <v>7.81562819139441</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="AK12" t="n">
         <v>38.15842840864836</v>
       </c>
-      <c r="AJ12" t="n">
+      <c r="AL12" t="n">
         <v>-80.45497299576715</v>
       </c>
-      <c r="AK12" t="n">
+      <c r="AM12" t="n">
         <v>-31.42346434456669</v>
       </c>
-      <c r="AL12" t="n">
+      <c r="AN12" t="n">
         <v>-0.3468083403687878</v>
       </c>
-      <c r="AM12" t="n">
+      <c r="AO12" t="n">
         <v>-25.83642864398556</v>
       </c>
     </row>
@@ -2023,69 +2099,75 @@
         <v>186.6376399803823</v>
       </c>
       <c r="R13" t="n">
+        <v>67.60161191421548</v>
+      </c>
+      <c r="S13" t="n">
         <v>30.86135953909287</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>39.95200070978618</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>2199.984</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>176.4447</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>68.863</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>85.12113720642769</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>178.7543881334982</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>1.013090153081947</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AA13" t="n">
         <v>765.7402</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>14.36205245897539</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>570.3287</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>3.232336817144408</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>1.638711519816756</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>0.14247457554881</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AG13" t="n">
         <v>546.0051999999999</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AH13" t="n">
         <v>114.9905340443179</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="AI13" t="n">
+        <v>74.71778220296761</v>
+      </c>
+      <c r="AJ13" t="n">
         <v>7.498332516326033</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AK13" t="n">
         <v>37.49644309680975</v>
       </c>
-      <c r="AJ13" t="n">
+      <c r="AL13" t="n">
         <v>-68.2338885370763</v>
       </c>
-      <c r="AK13" t="n">
+      <c r="AM13" t="n">
         <v>-27.62636731462547</v>
       </c>
-      <c r="AL13" t="n">
+      <c r="AN13" t="n">
         <v>-0.3581558227617399</v>
       </c>
-      <c r="AM13" t="n">
+      <c r="AO13" t="n">
         <v>-26.11900629581628</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Save combustion comparison workflow and outputs
</commit_message>
<xml_diff>
--- a/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
+++ b/out_FPT/compare_p241075_nef6_horsch_full_load_curve_sala01_puc_minas_d85b15__vs__p251122_nef67_175kw_mar_l_sn2040912_full_load_curve_rev24_e94h6.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO13"/>
+  <dimension ref="A1:AZ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,6 +622,61 @@
           <t>Economia_vs_Diesel_R_kWh_pct</t>
         </is>
       </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>E94H6_PCYL1</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>E94H6_APMAX1</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>E94H6_PMAX1</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>E94H6_IMEP1</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>E94H6_IMEPH1</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>E94H6_IMPEL1</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>E94H6_AI05_1</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>E94H6_AI10_1</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>E94H6_AI50_1</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>E94H6_AI90_1</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>E94H6_RMAX1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -751,6 +806,39 @@
       <c r="AO2" t="n">
         <v>-22.97036117831891</v>
       </c>
+      <c r="AP2" t="n">
+        <v>1.092622</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>18.09375</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>86.6759</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>16.68665</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>16.55026</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0.1332705</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>4.53125</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>6.304688</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>13.42188</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>22.74219</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>4.626417</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -880,6 +968,39 @@
       <c r="AO3" t="n">
         <v>-23.53862927536348</v>
       </c>
+      <c r="AP3" t="n">
+        <v>1.143285</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>88.6845</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>16.71579</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>16.6485</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>0.06401568000000001</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>3.8125</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>5.632813</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>12.74219</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>22.1875</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>4.902439</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1009,6 +1130,39 @@
       <c r="AO4" t="n">
         <v>-23.90102195316334</v>
       </c>
+      <c r="AP4" t="n">
+        <v>1.170852</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>17.67742</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>88.9072</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>16.97852</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>16.9824</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>-0.006760174</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>3.774194</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>5.653226</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>12.95968</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>22.64516</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>4.638342</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1138,6 +1292,39 @@
       <c r="AO5" t="n">
         <v>-23.65164175962884</v>
       </c>
+      <c r="AP5" t="n">
+        <v>1.241171</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>18.125</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>90.5236</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>17.46548</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>17.54554</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>-0.08268010000000001</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>4.179688</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>6.070313</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>13.375</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>23.0625</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>4.76997</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1267,6 +1454,39 @@
       <c r="AO6" t="n">
         <v>-25.19876706202729</v>
       </c>
+      <c r="AP6" t="n">
+        <v>1.379648</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>17.09375</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>98.05710000000001</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>18.18471</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>18.34434</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>-0.1617583</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>2.804688</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>4.671875</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>12.02344</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>21.625</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>5.12636</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1396,6 +1616,39 @@
       <c r="AO7" t="n">
         <v>-24.92231049108856</v>
       </c>
+      <c r="AP7" t="n">
+        <v>1.406529</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>16.5625</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>99.941</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>18.34892</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>18.61006</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>-0.2645763</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>2.40625</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>4.265625</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>11.67188</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>21.33594</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>5.188992</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1525,6 +1778,39 @@
       <c r="AO8" t="n">
         <v>-24.91302084088255</v>
       </c>
+      <c r="AP8" t="n">
+        <v>1.443125</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>15.6129</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>102.4589</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>18.30097</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>18.65453</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>-0.3554161</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>1.758065</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>3.572581</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>10.82258</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>20.48387</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>5.517722</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1654,6 +1940,39 @@
       <c r="AO9" t="n">
         <v>-25.36276139596612</v>
       </c>
+      <c r="AP9" t="n">
+        <v>1.479748</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>15.6129</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>99.089</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>17.49736</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>17.95029</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>-0.4551287</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>1.564516</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>3.403226</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>10.6371</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>20.54839</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>5.406726</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1783,6 +2102,39 @@
       <c r="AO10" t="n">
         <v>-26.11364120894262</v>
       </c>
+      <c r="AP10" t="n">
+        <v>1.471356</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>15.48387</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>96.5155</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>17.03395</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>17.56327</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>-0.5313497</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>1.354839</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>3.217742</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>10.6371</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>20.84678</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>5.17787</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1912,6 +2264,39 @@
       <c r="AO11" t="n">
         <v>-27.67694168890273</v>
       </c>
+      <c r="AP11" t="n">
+        <v>1.499267</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>15.32258</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>94.8122</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>16.34813</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>16.9584</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>-0.6126408</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.895161</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>2.758065</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>10.15323</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>19.96774</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>5.130383</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2041,6 +2426,39 @@
       <c r="AO12" t="n">
         <v>-25.83642864398556</v>
       </c>
+      <c r="AP12" t="n">
+        <v>1.492086</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>14.875</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>91.02849999999999</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>15.39127</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>16.07301</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>-0.6846895</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>2.375</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>9.664059999999999</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>5.037124</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2169,6 +2587,39 @@
       </c>
       <c r="AO13" t="n">
         <v>-26.11900629581628</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>1.518564</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>14.51515</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>89.0171</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>14.8104</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>15.57817</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>-0.7704704</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0.0984849</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>1.969697</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>9.257580000000001</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>19.29545</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>5.038199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>